<commit_message>
Enforce strict 2-attempt order limit per customer (Phone/Device/IP) across storefront and backend risk engine
</commit_message>
<xml_diff>
--- a/data/excel/Orders.xlsx
+++ b/data/excel/Orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Y11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1092,9 +1092,163 @@
         <v>2026-08-21T15:26:27.155Z</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TEST-001</v>
+      </c>
+      <c r="B10" t="str">
+        <v>yamahasac</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="D10" t="str">
+        <v>0770998877</v>
+      </c>
+      <c r="E10" t="str">
+        <v>16 - Alger</v>
+      </c>
+      <c r="F10" t="str">
+        <v>الجزائر</v>
+      </c>
+      <c r="G10" t="str">
+        <v>توصيل للمنزل</v>
+      </c>
+      <c r="H10" t="str">
+        <v>24 - 48 H</v>
+      </c>
+      <c r="I10" t="str">
+        <v>1</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Sac Banane Moto Yamaha (كرطابل يماها)</v>
+      </c>
+      <c r="K10" t="str">
+        <v>3900 د.ج</v>
+      </c>
+      <c r="L10" t="str">
+        <v>500 د.ج</v>
+      </c>
+      <c r="M10" t="str">
+        <v>3900</v>
+      </c>
+      <c r="N10" t="str">
+        <v>3900 د.ج</v>
+      </c>
+      <c r="O10" t="str">
+        <v>deleted</v>
+      </c>
+      <c r="P10" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v>[]</v>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v>0</v>
+      </c>
+      <c r="V10" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="W10" t="str">
+        <v>ALLOW</v>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v>2026-08-21T18:23:28.323Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TEST-002</v>
+      </c>
+      <c r="B11" t="str">
+        <v>yamahasac</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0770998877</v>
+      </c>
+      <c r="E11" t="str">
+        <v>16 - Alger</v>
+      </c>
+      <c r="F11" t="str">
+        <v>الجزائر</v>
+      </c>
+      <c r="G11" t="str">
+        <v>توصيل للمنزل</v>
+      </c>
+      <c r="H11" t="str">
+        <v>24 - 48 H</v>
+      </c>
+      <c r="I11" t="str">
+        <v>1</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Sac Banane Moto Yamaha (كرطابل يماها)</v>
+      </c>
+      <c r="K11" t="str">
+        <v>3900 د.ج</v>
+      </c>
+      <c r="L11" t="str">
+        <v>500 د.ج</v>
+      </c>
+      <c r="M11" t="str">
+        <v>3900</v>
+      </c>
+      <c r="N11" t="str">
+        <v>3900 د.ج</v>
+      </c>
+      <c r="O11" t="str">
+        <v>deleted</v>
+      </c>
+      <c r="P11" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v>[]</v>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v>0</v>
+      </c>
+      <c r="V11" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="W11" t="str">
+        <v>ALLOW</v>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v>2026-08-21T18:23:28.416Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: connect Supabase PostgreSQL, fix communes dropdown, add admin password gate & mobile-first orders view, rebrand store to ORVA STORE
</commit_message>
<xml_diff>
--- a/data/excel/Orders.xlsx
+++ b/data/excel/Orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1323,9 +1323,86 @@
         <v>2026-10-05T17:49:22.348Z</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TEST-ORVA-1791233238380</v>
+      </c>
+      <c r="B13" t="str">
+        <v>orvastore</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Mohamed Amine</v>
+      </c>
+      <c r="D13" t="str">
+        <v>0661998877</v>
+      </c>
+      <c r="E13" t="str">
+        <v>07 - بسكرة</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Biskra</v>
+      </c>
+      <c r="G13" t="str">
+        <v>توصيل للمنزل</v>
+      </c>
+      <c r="H13" t="str">
+        <v>24 - 48 H</v>
+      </c>
+      <c r="I13" t="str">
+        <v>1</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Pack 1 Pro (4 أدوات)</v>
+      </c>
+      <c r="K13" t="str">
+        <v>4950 د.ج</v>
+      </c>
+      <c r="L13" t="str">
+        <v>500 د.ج</v>
+      </c>
+      <c r="M13" t="str">
+        <v>4950</v>
+      </c>
+      <c r="N13" t="str">
+        <v>5450 د.ج</v>
+      </c>
+      <c r="O13" t="str">
+        <v>deleted</v>
+      </c>
+      <c r="P13" t="str">
+        <v>false</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v>[]</v>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v>10</v>
+      </c>
+      <c r="V13" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="W13" t="str">
+        <v>ALLOW</v>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v>2026-10-05T20:47:18.914Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>